<commit_message>
Verify security-questionnaire kit and link it from its niche
Set up with kits/setup.sh, the sample commands rebuild the draft
library, the library check passes, the fill finds all 40 questions
(15 OK, 18 CHECK, 7 NEEDS CLIENT INPUT) and finalising refuses while
review items remain.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DspfyLwNfeJ4CHdyACeRHQ
</commit_message>
<xml_diff>
--- a/kits/security-questionnaire/samples/library/answer_library.xlsx
+++ b/kits/security-questionnaire/samples/library/answer_library.xlsx
@@ -27,10 +27,10 @@
   </numFmts>
   <fonts count="4">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>

</xml_diff>